<commit_message>
Fix prefetch: single cron + market hours in Python + keepalive
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD00FC47-AD74-4874-8341-42C7F862E4B6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
   <si>
     <t>Ticker</t>
   </si>
@@ -219,6 +219,12 @@
   </si>
   <si>
     <t>CHRW</t>
+  </si>
+  <si>
+    <t>AXP</t>
+  </si>
+  <si>
+    <t>DELL</t>
   </si>
 </sst>
 </file>
@@ -280,12 +286,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -704,7 +711,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A63"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1025,12 +1032,45 @@
         <v>64</v>
       </c>
     </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1243,37 +1283,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists 2026-04-21 06:53
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD00FC47-AD74-4874-8341-42C7F862E4B6}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75EB95F6-4813-4A44-8510-E3522B2981FF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>Ticker</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>DELL</t>
+  </si>
+  <si>
+    <t>DOX</t>
   </si>
 </sst>
 </file>
@@ -292,7 +295,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -702,7 +705,9 @@
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1062,15 +1067,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1283,6 +1279,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
   <ds:schemaRefs>
@@ -1295,14 +1300,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1319,4 +1316,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-06-03 09:20
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44F8F0B6-8142-4ABC-A310-4A9C2559DF07}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56AF7C3F-5FC7-41D4-B1F2-AFA3081840FB}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
   <si>
     <t>Ticker</t>
   </si>
@@ -192,9 +192,6 @@
   </si>
   <si>
     <t>LRCX</t>
-  </si>
-  <si>
-    <t>PEG</t>
   </si>
   <si>
     <t>FIX</t>
@@ -724,7 +721,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1017,12 +1014,12 @@
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>4</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
@@ -1041,7 +1038,7 @@
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
+      <c r="A63" s="3" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1063,11 +1060,6 @@
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1085,6 +1077,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1297,20 +1303,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
@@ -1320,6 +1312,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1336,15 +1339,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-06-09 10:09
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56AF7C3F-5FC7-41D4-B1F2-AFA3081840FB}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F44D74CC-CF15-4BA9-A006-7E07699BA7E7}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
   <si>
     <t>Ticker</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t>LII</t>
+  </si>
+  <si>
+    <t>NVDA</t>
   </si>
 </sst>
 </file>
@@ -721,7 +724,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A67"/>
+  <dimension ref="A1:A68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1062,6 +1065,11 @@
         <v>68</v>
       </c>
     </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1077,20 +1085,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1303,6 +1297,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
@@ -1312,17 +1320,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1339,4 +1336,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-06-18 14:07
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F44D74CC-CF15-4BA9-A006-7E07699BA7E7}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF1D1890-7332-4810-9F60-797AF8A33A0C}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
   <si>
     <t>Ticker</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>NVDA</t>
+  </si>
+  <si>
+    <t>ACM</t>
   </si>
 </sst>
 </file>
@@ -680,7 +683,7 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>5</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -1085,6 +1088,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1297,20 +1314,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
@@ -1320,6 +1323,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1336,15 +1350,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Watchlists (Watchlists.xlsx) 2026-07-14 09:31
</commit_message>
<xml_diff>
--- a/data/Watchlists.xlsx
+++ b/data/Watchlists.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://martincp1.sharepoint.com/sites/Eugene/Shared Documents/Operations/Scripts/Portfolio Dashboard/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF1D1890-7332-4810-9F60-797AF8A33A0C}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{0BBD03A5-0612-494C-9327-617BBDD1F095}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8246B333-F41A-482E-89AE-B3C7B6FC1C48}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="QDVD Watchlist A" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="72">
   <si>
     <t>Ticker</t>
   </si>
@@ -237,6 +237,9 @@
   </si>
   <si>
     <t>ACM</t>
+  </si>
+  <si>
+    <t>WSO</t>
   </si>
 </sst>
 </file>
@@ -727,7 +730,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1073,6 +1076,11 @@
         <v>69</v>
       </c>
     </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1088,20 +1096,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100816A82F3E39F6D48966CE5F2A60D183C" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ee6fa4220ecdfcc2f6fea1f3e0d62b76">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="db58b361-de72-439a-9b19-5afb42a4fe9e" xmlns:ns3="e26837be-2e64-4fb1-8d10-81cb111b0084" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54ce9d38be15445670b4f969d736cc65" ns2:_="" ns3:_="">
     <xsd:import namespace="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
@@ -1314,6 +1308,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdPermissions xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <TaxCatchAll xmlns="e26837be-2e64-4fb1-8d10-81cb111b0084" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizId xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+    <MigrationWizIdVersion xmlns="db58b361-de72-439a-9b19-5afb42a4fe9e" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54F23C73-979C-443E-9CA2-7121B6C69145}">
   <ds:schemaRefs>
@@ -1323,17 +1331,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
-    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A7D093A-965A-49F4-B796-FB43CAA20C7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1350,4 +1347,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D745EAF-ECE4-4450-8AD0-64918CC3B71B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="db58b361-de72-439a-9b19-5afb42a4fe9e"/>
+    <ds:schemaRef ds:uri="e26837be-2e64-4fb1-8d10-81cb111b0084"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>